<commit_message>
Fetch licensed car photos from Wikimedia Commons
</commit_message>
<xml_diff>
--- a/content/cars.xlsx
+++ b/content/cars.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="358">
   <si>
     <t>طريقة تحديث سيارات الموقع</t>
   </si>
@@ -267,6 +267,9 @@
     <t>شاشة 9 بوصة، آبل كاربلاي وأندرويد أوتو، كاميرا خلفية، مثبت سرعة تكيفي، نظام Toyota Safety Sense، مقاعد رياضية، تشغيل بدون مفتاح</t>
   </si>
   <si>
+    <t>car-001-1.webp، car-001-2.webp، car-001-3.webp</t>
+  </si>
+  <si>
     <t>car-002</t>
   </si>
   <si>
@@ -291,6 +294,9 @@
     <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، مثبت سرعة تكيفي، تنبيه مغادرة المسار، جنوط 18 بوصة</t>
   </si>
   <si>
+    <t>car-002-1.webp، car-002-2.webp، car-002-3.webp</t>
+  </si>
+  <si>
     <t>car-003</t>
   </si>
   <si>
@@ -327,6 +333,9 @@
     <t>دفع رباعي دائم مع قفل تفاضلي، شاشة 12.3 بوصة، كاميرا 360 درجة، مقاعد جلد كهربائية، فتحة سقف، سبعة مقاعد، مثبت سرعة تكيفي</t>
   </si>
   <si>
+    <t>car-003-1.webp، car-003-2.webp، car-003-3.webp</t>
+  </si>
+  <si>
     <t>car-004</t>
   </si>
   <si>
@@ -351,6 +360,9 @@
     <t>دفع رباعي، سبعة مقاعد، مقاعد جلد، شاشة وسطية، كاميرا خلفية، حساسات ركن أمامية وخلفية</t>
   </si>
   <si>
+    <t>car-004-1.webp، car-004-2.webp، car-004-3.webp</t>
+  </si>
+  <si>
     <t>car-005</t>
   </si>
   <si>
@@ -378,6 +390,9 @@
     <t>شاشة بانورامية مزدوجة، مقاعد جلد مهواة، شاحن لاسلكي، كاميرا خلفية، تحكم مناخي ثنائي، بصمة تشغيل</t>
   </si>
   <si>
+    <t>car-005-1.webp، car-005-2.webp، car-005-3.webp</t>
+  </si>
+  <si>
     <t>car-006</t>
   </si>
   <si>
@@ -393,6 +408,9 @@
     <t>شاشة منحنية مزدوجة 12.3 بوصة، فتحة سقف بانورامية، كاميرا خلفية، حساسات ركن، مقاعد جلد، شاحن لاسلكي</t>
   </si>
   <si>
+    <t>car-006-1.webp، car-006-2.webp، car-006-3.webp</t>
+  </si>
+  <si>
     <t>car-007</t>
   </si>
   <si>
@@ -414,6 +432,9 @@
     <t>سبعة مقاعد، دفع كلي AWD، شاشة 12.3 بوصة، كاميرا 360 درجة، مقاعد جلد، فتحة سقف بانورامية، ضمان الوكيل</t>
   </si>
   <si>
+    <t>car-007-1.webp، car-007-2.webp، car-007-3.webp</t>
+  </si>
+  <si>
     <t>car-008</t>
   </si>
   <si>
@@ -429,6 +450,9 @@
     <t>شاشة 10.25 بوصة، كاميرا خلفية، بلوتوث، تحكم مناخي، مقاعد مدفأة</t>
   </si>
   <si>
+    <t>car-008-1.webp، car-008-2.webp، car-008-3.webp</t>
+  </si>
+  <si>
     <t>car-009</t>
   </si>
   <si>
@@ -444,6 +468,9 @@
     <t>شاشة 12.3 بوصة، كاميرا خلفية، حساسات ركن، مقاعد جلد، تحكم مناخي أوتوماتيك، مثبت سرعة</t>
   </si>
   <si>
+    <t>car-009-1.webp، car-009-2.webp، car-009-3.webp</t>
+  </si>
+  <si>
     <t>car-010</t>
   </si>
   <si>
@@ -462,6 +489,9 @@
     <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، مثبت سرعة، تنبيه النقطة العمياء</t>
   </si>
   <si>
+    <t>car-010-1.webp، car-010-2.webp</t>
+  </si>
+  <si>
     <t>car-011</t>
   </si>
   <si>
@@ -483,6 +513,9 @@
     <t>شاشة 8 بوصة، كاميرا خلفية، مثبت سرعة تكيفي ProPilot، مقاعد مدفأة، تشغيل بدون مفتاح</t>
   </si>
   <si>
+    <t>car-011-1.webp، car-011-2.webp، car-011-3.webp</t>
+  </si>
+  <si>
     <t>car-012</t>
   </si>
   <si>
@@ -498,6 +531,9 @@
     <t>شاشتان 14.3 بوصة، كاميرا 360 درجة، تعليق هوائي، مقاعد جلد مدفأة ومهواة، نظام صوت Klipsch، فتحة سقف بانورامية، ثمانية مقاعد</t>
   </si>
   <si>
+    <t>car-012-1.webp، car-012-2.webp، car-012-3.webp</t>
+  </si>
+  <si>
     <t>car-013</t>
   </si>
   <si>
@@ -516,6 +552,9 @@
     <t>شاشة وسطية، بلوتوث، كاميرا خلفية، مكيف أوتوماتيك</t>
   </si>
   <si>
+    <t>car-013-1.webp، car-013-2.webp، car-013-3.webp</t>
+  </si>
+  <si>
     <t>car-014</t>
   </si>
   <si>
@@ -537,6 +576,9 @@
     <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، تشغيل عن بعد، مقاعد قماش فاخر</t>
   </si>
   <si>
+    <t>car-014-1.webp، car-014-2.webp</t>
+  </si>
+  <si>
     <t>car-015</t>
   </si>
   <si>
@@ -552,6 +594,9 @@
     <t>ثمانية مقاعد، دفع رباعي، شاشة 10.2 بوصة، مقاعد جلد، كاميرا خلفية، تشغيل عن بعد</t>
   </si>
   <si>
+    <t>car-015-1.webp، car-015-2.webp، car-015-3.webp</t>
+  </si>
+  <si>
     <t>car-016</t>
   </si>
   <si>
@@ -567,6 +612,9 @@
     <t>مقاعد جلد مدفأة ومهواة، فتحة سقف، نظام صوت مارك ليفنسون، شاشة 12.3 بوصة، كاميرا خلفية، حساسات ركن</t>
   </si>
   <si>
+    <t>car-016-1.webp، car-016-2.webp، car-016-3.webp</t>
+  </si>
+  <si>
     <t>car-017</t>
   </si>
   <si>
@@ -585,6 +633,9 @@
     <t>شاشة 14 بوصة، مقاعد جلد، فتحة سقف بانورامية، كاميرا 360 درجة، دفع كلي AWD، مثبت سرعة تكيفي</t>
   </si>
   <si>
+    <t>car-017-1.webp، car-017-2.webp، car-017-3.webp</t>
+  </si>
+  <si>
     <t>car-018</t>
   </si>
   <si>
@@ -609,6 +660,9 @@
     <t>شاشة MBUX 11.9 بوصة، مقاعد جلد مدفأة، كاميرا 360 درجة، إضاءة أمبيانت، فتحة سقف بانورامية</t>
   </si>
   <si>
+    <t>car-018-1.webp، car-018-2.webp، car-018-3.webp</t>
+  </si>
+  <si>
     <t>car-019</t>
   </si>
   <si>
@@ -627,6 +681,9 @@
     <t>تعليق هوائي، مقاعد جلد نابا، فتحة سقف بانورامية، شاشتان MBUX، كاميرا 360 درجة، نظام صوت Burmester</t>
   </si>
   <si>
+    <t>car-019-1.webp، car-019-2.webp، car-019-3.webp</t>
+  </si>
+  <si>
     <t>car-020</t>
   </si>
   <si>
@@ -645,6 +702,9 @@
     <t>شاشة منحنية iDrive 8.5، مقاعد جلد رياضية، كاميرا خلفية، مثبت سرعة تكيفي، شاحن لاسلكي، ضمان الوكيل</t>
   </si>
   <si>
+    <t>car-020-1.webp، car-020-2.webp، car-020-3.webp</t>
+  </si>
+  <si>
     <t>car-021</t>
   </si>
   <si>
@@ -663,6 +723,9 @@
     <t>مقاعد جلد ميرينو، فتحة سقف بانورامية، كاميرا 360 درجة، نظام صوت هارمان كاردون، دفع كلي xDrive، تعليق هوائي</t>
   </si>
   <si>
+    <t>car-021-1.webp، car-021-2.webp، car-021-3.webp</t>
+  </si>
+  <si>
     <t>car-022</t>
   </si>
   <si>
@@ -684,6 +747,9 @@
     <t>سبعة مقاعد، دفع رباعي، شاشة 8 بوصة، كاميرا خلفية، حساسات ركن، مقاعد كهربائية</t>
   </si>
   <si>
+    <t>car-022-1.webp، car-022-2.webp، car-022-3.webp</t>
+  </si>
+  <si>
     <t>car-023</t>
   </si>
   <si>
@@ -702,6 +768,9 @@
     <t>دفع كلي مع تعليق هوائي، شاشة Pivi Pro 11.4 بوصة، كاميرا 360 درجة، مقاعد جلد، نظام Terrain Response</t>
   </si>
   <si>
+    <t>car-023-1.webp، car-023-2.webp، car-023-3.webp</t>
+  </si>
+  <si>
     <t>car-024</t>
   </si>
   <si>
@@ -720,6 +789,9 @@
     <t>شاشة 8 بوصة، بلوتوث، كاميرا خلفية، مكيف</t>
   </si>
   <si>
+    <t>car-024-1.webp، car-024-2.webp، car-024-3.webp</t>
+  </si>
+  <si>
     <t>car-025</t>
   </si>
   <si>
@@ -744,6 +816,9 @@
     <t>محرك كهربائي مزدوج AWD، شحن فائق السرعة 800 فولت، شاشة بانورامية مزدوجة، مساعد قيادة ذكي، مقاعد جلد نباتي</t>
   </si>
   <si>
+    <t>car-025-1.webp، car-025-2.webp، car-025-3.webp</t>
+  </si>
+  <si>
     <t>car-026</t>
   </si>
   <si>
@@ -762,6 +837,9 @@
     <t>نظام هجين 225 حصان، شاشة 12.3 بوصة، آبل كاربلاي لاسلكي، كاميرا خلفية، Toyota Safety Sense 3.0، مقاعد رياضية</t>
   </si>
   <si>
+    <t>car-026-1.webp، car-026-2.webp، car-026-3.webp</t>
+  </si>
+  <si>
     <t>car-027</t>
   </si>
   <si>
@@ -780,6 +858,9 @@
     <t>شاشة 7 بوصة، آبل كاربلاي، كاميرا خلفية، جنوط رياضية 18 بوصة، نظام Honda Sensing</t>
   </si>
   <si>
+    <t>car-027-1.webp، car-027-2.webp، car-027-3.webp</t>
+  </si>
+  <si>
     <t>car-028</t>
   </si>
   <si>
@@ -801,6 +882,9 @@
     <t>دفع رباعي Super Select، سبعة مقاعد، شاشة وسطية، كاميرا خلفية، مقاعد جلد</t>
   </si>
   <si>
+    <t>car-028-1.webp، car-028-2.webp، car-028-3.webp</t>
+  </si>
+  <si>
     <t>car-029</t>
   </si>
   <si>
@@ -822,6 +906,9 @@
     <t>دفع رباعي، صندوق خلفي، شاشة 8 بوصة، كاميرا خلفية، مثبت سرعة</t>
   </si>
   <si>
+    <t>car-029-1.webp، car-029-2.webp، car-029-3.webp</t>
+  </si>
+  <si>
     <t>car-030</t>
   </si>
   <si>
@@ -837,6 +924,9 @@
     <t>شاشتان 12.3 بوصة، كاميرا 360 درجة، فتحة سقف بانورامية، مقاعد جلد كهربائية، شاحن لاسلكي، ضمان الوكيل</t>
   </si>
   <si>
+    <t>car-030-1.webp، car-030-2.webp، car-030-3.webp</t>
+  </si>
+  <si>
     <t>car-031</t>
   </si>
   <si>
@@ -852,6 +942,9 @@
     <t>شاشة 10.25 بوصة، كاميرا 360 درجة، فتحة سقف، مثبت سرعة تكيفي، ضمان الوكيل</t>
   </si>
   <si>
+    <t>car-031-1.webp، car-031-2.webp، car-031-3.webp</t>
+  </si>
+  <si>
     <t>car-032</t>
   </si>
   <si>
@@ -867,6 +960,9 @@
     <t>شاشة 12.3 بوصة، كاميرا 360 درجة، فتحة سقف بانورامية، مقاعد جلد، شاحن لاسلكي، ركن ذاتي</t>
   </si>
   <si>
+    <t>car-032-1.webp، car-032-2.webp</t>
+  </si>
+  <si>
     <t>car-033</t>
   </si>
   <si>
@@ -885,6 +981,9 @@
     <t>سبعة مقاعد، دفع كلي HTRAC، شاشة بانورامية مزدوجة، كاميرا 360 درجة، مقاعد جلد مهواة، شاحن لاسلكي مزدوج</t>
   </si>
   <si>
+    <t>car-033-1.webp، car-033-2.webp، car-033-3.webp</t>
+  </si>
+  <si>
     <t>car-034</t>
   </si>
   <si>
@@ -898,6 +997,9 @@
   </si>
   <si>
     <t>سبعة مقاعد، دفع كلي، شاشتان 12.3 بوصة، كاميرا 360 درجة، مقاعد جلد كهربائية مدفأة، نظام صوت Sony</t>
+  </si>
+  <si>
+    <t>car-034-1.webp، car-034-2.webp</t>
   </si>
   <si>
     <t>الحالة</t>
@@ -1863,17 +1965,19 @@
       <c r="X2" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="Y2" s="7"/>
+      <c r="Y2" s="7" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>69</v>
@@ -1903,7 +2007,7 @@
         <v>74</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N3" s="7">
         <v>4</v>
@@ -1918,10 +2022,10 @@
         <v>5</v>
       </c>
       <c r="R3" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S3" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="T3" s="7" t="s">
         <v>79</v>
@@ -1930,28 +2034,30 @@
         <v>80</v>
       </c>
       <c r="V3" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W3" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="X3" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="Y3" s="7"/>
+        <v>91</v>
+      </c>
+      <c r="Y3" s="7" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E4" s="7">
         <v>2026</v>
@@ -1960,13 +2066,13 @@
         <v>135000000</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J4" s="8">
         <v>0</v>
@@ -1978,7 +2084,7 @@
         <v>74</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="N4" s="7">
         <v>6</v>
@@ -1987,13 +2093,13 @@
         <v>409</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q4" s="7">
         <v>7</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S4" s="7" t="s">
         <v>78</v>
@@ -2005,28 +2111,30 @@
         <v>80</v>
       </c>
       <c r="V4" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W4" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="X4" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="Y4" s="7"/>
+        <v>104</v>
+      </c>
+      <c r="Y4" s="7" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E5" s="7">
         <v>2023</v>
@@ -2038,10 +2146,10 @@
         <v>70</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J5" s="8">
         <v>38000</v>
@@ -2053,7 +2161,7 @@
         <v>74</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="N5" s="7">
         <v>6</v>
@@ -2062,16 +2170,16 @@
         <v>271</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q5" s="7">
         <v>7</v>
       </c>
       <c r="R5" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="S5" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="T5" s="7" t="s">
         <v>79</v>
@@ -2079,25 +2187,27 @@
       <c r="U5" s="7"/>
       <c r="V5" s="7"/>
       <c r="W5" s="9" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="X5" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="Y5" s="7"/>
+        <v>113</v>
+      </c>
+      <c r="Y5" s="7" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E6" s="7">
         <v>2024</v>
@@ -2109,7 +2219,7 @@
         <v>70</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>72</v>
@@ -2124,7 +2234,7 @@
         <v>74</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="N6" s="7">
         <v>4</v>
@@ -2139,7 +2249,7 @@
         <v>5</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>78</v>
@@ -2152,25 +2262,27 @@
       </c>
       <c r="V6" s="7"/>
       <c r="W6" s="9" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="X6" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="Y6" s="7"/>
+        <v>123</v>
+      </c>
+      <c r="Y6" s="7" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E7" s="7">
         <v>2023</v>
@@ -2182,10 +2294,10 @@
         <v>70</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J7" s="8">
         <v>27000</v>
@@ -2197,7 +2309,7 @@
         <v>74</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="N7" s="7">
         <v>4</v>
@@ -2212,10 +2324,10 @@
         <v>5</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S7" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="T7" s="7" t="s">
         <v>79</v>
@@ -2225,22 +2337,24 @@
       </c>
       <c r="V7" s="7"/>
       <c r="W7" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="X7" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="Y7" s="7"/>
+        <v>129</v>
+      </c>
+      <c r="Y7" s="7" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7">
@@ -2250,13 +2364,13 @@
         <v>58000000</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H8" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I8" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
@@ -2268,7 +2382,7 @@
         <v>74</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="N8" s="7">
         <v>6</v>
@@ -2277,13 +2391,13 @@
         <v>272</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q8" s="7">
         <v>7</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="S8" s="7" t="s">
         <v>78</v>
@@ -2294,22 +2408,24 @@
       <c r="U8" s="7"/>
       <c r="V8" s="7"/>
       <c r="W8" s="9" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="X8" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y8" s="7"/>
+        <v>137</v>
+      </c>
+      <c r="Y8" s="7" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7">
@@ -2322,7 +2438,7 @@
         <v>70</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>72</v>
@@ -2352,7 +2468,7 @@
         <v>5</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S9" s="7" t="s">
         <v>78</v>
@@ -2363,22 +2479,24 @@
       <c r="U9" s="7"/>
       <c r="V9" s="7"/>
       <c r="W9" s="9" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="X9" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="Y9" s="7"/>
+        <v>143</v>
+      </c>
+      <c r="Y9" s="7" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7">
@@ -2391,10 +2509,10 @@
         <v>70</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J10" s="8">
         <v>14000</v>
@@ -2406,7 +2524,7 @@
         <v>74</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N10" s="7">
         <v>4</v>
@@ -2421,10 +2539,10 @@
         <v>5</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S10" s="7" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="T10" s="7" t="s">
         <v>79</v>
@@ -2434,25 +2552,27 @@
       </c>
       <c r="V10" s="7"/>
       <c r="W10" s="9" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="X10" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="Y10" s="7"/>
+        <v>149</v>
+      </c>
+      <c r="Y10" s="7" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="E11" s="7">
         <v>2023</v>
@@ -2479,7 +2599,7 @@
         <v>74</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N11" s="7">
         <v>4</v>
@@ -2494,38 +2614,40 @@
         <v>5</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="S11" s="7" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="T11" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U11" s="7"/>
       <c r="V11" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W11" s="9" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="X11" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="Y11" s="7"/>
+        <v>156</v>
+      </c>
+      <c r="Y11" s="7" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="E12" s="7">
         <v>2023</v>
@@ -2567,36 +2689,38 @@
         <v>5</v>
       </c>
       <c r="R12" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S12" s="7" t="s">
         <v>78</v>
       </c>
       <c r="T12" s="7" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="U12" s="7"/>
       <c r="V12" s="7"/>
       <c r="W12" s="9" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="X12" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="Y12" s="7"/>
+        <v>164</v>
+      </c>
+      <c r="Y12" s="7" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="E13" s="7">
         <v>2026</v>
@@ -2605,13 +2729,13 @@
         <v>160000000</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J13" s="8">
         <v>0</v>
@@ -2623,7 +2747,7 @@
         <v>74</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="N13" s="7">
         <v>6</v>
@@ -2632,13 +2756,13 @@
         <v>425</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q13" s="7">
         <v>8</v>
       </c>
       <c r="R13" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S13" s="7" t="s">
         <v>78</v>
@@ -2650,25 +2774,27 @@
         <v>80</v>
       </c>
       <c r="V13" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W13" s="9" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="X13" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="Y13" s="7"/>
+        <v>170</v>
+      </c>
+      <c r="Y13" s="7" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="7">
@@ -2681,7 +2807,7 @@
         <v>70</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>72</v>
@@ -2696,7 +2822,7 @@
         <v>74</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="N14" s="7">
         <v>4</v>
@@ -2711,38 +2837,40 @@
         <v>5</v>
       </c>
       <c r="R14" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S14" s="7" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="T14" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U14" s="7"/>
       <c r="V14" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W14" s="9" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="X14" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="Y14" s="7"/>
+        <v>177</v>
+      </c>
+      <c r="Y14" s="7" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="E15" s="7">
         <v>2023</v>
@@ -2769,7 +2897,7 @@
         <v>74</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="N15" s="7">
         <v>4</v>
@@ -2784,7 +2912,7 @@
         <v>5</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="S15" s="7" t="s">
         <v>78</v>
@@ -2797,25 +2925,27 @@
       </c>
       <c r="V15" s="7"/>
       <c r="W15" s="9" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="X15" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y15" s="7"/>
+        <v>185</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="E16" s="7">
         <v>2023</v>
@@ -2830,7 +2960,7 @@
         <v>71</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J16" s="8">
         <v>33000</v>
@@ -2842,7 +2972,7 @@
         <v>74</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="N16" s="7">
         <v>8</v>
@@ -2851,41 +2981,43 @@
         <v>355</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q16" s="7">
         <v>8</v>
       </c>
       <c r="R16" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S16" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="T16" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U16" s="7"/>
       <c r="V16" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W16" s="9" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="X16" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="Y16" s="7"/>
+        <v>191</v>
+      </c>
+      <c r="Y16" s="7" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="7">
@@ -2913,7 +3045,7 @@
         <v>74</v>
       </c>
       <c r="M17" s="7" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="N17" s="7">
         <v>6</v>
@@ -2928,7 +3060,7 @@
         <v>5</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S17" s="7" t="s">
         <v>78</v>
@@ -2940,25 +3072,27 @@
         <v>80</v>
       </c>
       <c r="V17" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W17" s="9" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="X17" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="Y17" s="7"/>
+        <v>197</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="7">
@@ -2971,10 +3105,10 @@
         <v>70</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J18" s="8">
         <v>15000</v>
@@ -2986,7 +3120,7 @@
         <v>74</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
       <c r="N18" s="7">
         <v>4</v>
@@ -2995,44 +3129,46 @@
         <v>275</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q18" s="7">
         <v>5</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="T18" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U18" s="7"/>
       <c r="V18" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W18" s="9" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
       <c r="X18" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="Y18" s="7"/>
+        <v>204</v>
+      </c>
+      <c r="Y18" s="7" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="E19" s="7">
         <v>2024</v>
@@ -3059,7 +3195,7 @@
         <v>74</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="N19" s="7">
         <v>4</v>
@@ -3068,13 +3204,13 @@
         <v>255</v>
       </c>
       <c r="P19" s="7" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="Q19" s="7">
         <v>5</v>
       </c>
       <c r="R19" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S19" s="7" t="s">
         <v>78</v>
@@ -3086,28 +3222,30 @@
         <v>80</v>
       </c>
       <c r="V19" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W19" s="9" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="X19" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="Y19" s="7"/>
+        <v>213</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="E20" s="7">
         <v>2026</v>
@@ -3116,13 +3254,13 @@
         <v>155000000</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J20" s="8">
         <v>0</v>
@@ -3134,7 +3272,7 @@
         <v>74</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="N20" s="7">
         <v>6</v>
@@ -3143,13 +3281,13 @@
         <v>375</v>
       </c>
       <c r="P20" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q20" s="7">
         <v>5</v>
       </c>
       <c r="R20" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="S20" s="7" t="s">
         <v>78</v>
@@ -3161,28 +3299,30 @@
         <v>80</v>
       </c>
       <c r="V20" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W20" s="9" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="X20" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="Y20" s="7"/>
+        <v>220</v>
+      </c>
+      <c r="Y20" s="7" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
       <c r="E21" s="7">
         <v>2026</v>
@@ -3191,10 +3331,10 @@
         <v>91000000</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>72</v>
@@ -3209,7 +3349,7 @@
         <v>74</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="N21" s="7">
         <v>4</v>
@@ -3218,16 +3358,16 @@
         <v>208</v>
       </c>
       <c r="P21" s="7" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="Q21" s="7">
         <v>5</v>
       </c>
       <c r="R21" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S21" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="T21" s="7" t="s">
         <v>79</v>
@@ -3236,28 +3376,30 @@
         <v>80</v>
       </c>
       <c r="V21" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W21" s="9" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="X21" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="Y21" s="7"/>
+        <v>227</v>
+      </c>
+      <c r="Y21" s="7" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>209</v>
+        <v>229</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>211</v>
+        <v>231</v>
       </c>
       <c r="E22" s="7">
         <v>2026</v>
@@ -3266,13 +3408,13 @@
         <v>135000000</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J22" s="8">
         <v>0</v>
@@ -3284,7 +3426,7 @@
         <v>74</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>212</v>
+        <v>232</v>
       </c>
       <c r="N22" s="7">
         <v>6</v>
@@ -3293,13 +3435,13 @@
         <v>375</v>
       </c>
       <c r="P22" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q22" s="7">
         <v>5</v>
       </c>
       <c r="R22" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S22" s="7" t="s">
         <v>78</v>
@@ -3311,28 +3453,30 @@
         <v>80</v>
       </c>
       <c r="V22" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W22" s="9" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="X22" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="Y22" s="7"/>
+        <v>234</v>
+      </c>
+      <c r="Y22" s="7" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="E23" s="7">
         <v>2022</v>
@@ -3347,7 +3491,7 @@
         <v>71</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J23" s="8">
         <v>58000</v>
@@ -3359,7 +3503,7 @@
         <v>74</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="N23" s="7">
         <v>4</v>
@@ -3368,13 +3512,13 @@
         <v>300</v>
       </c>
       <c r="P23" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q23" s="7">
         <v>7</v>
       </c>
       <c r="R23" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S23" s="7" t="s">
         <v>78</v>
@@ -3385,25 +3529,27 @@
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
       <c r="W23" s="9" t="s">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="X23" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="Y23" s="7"/>
+        <v>242</v>
+      </c>
+      <c r="Y23" s="7" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>223</v>
+        <v>245</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>224</v>
+        <v>246</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>225</v>
+        <v>247</v>
       </c>
       <c r="E24" s="7">
         <v>2024</v>
@@ -3415,10 +3561,10 @@
         <v>70</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J24" s="8">
         <v>12000</v>
@@ -3430,7 +3576,7 @@
         <v>74</v>
       </c>
       <c r="M24" s="7" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="N24" s="7">
         <v>6</v>
@@ -3439,16 +3585,16 @@
         <v>395</v>
       </c>
       <c r="P24" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q24" s="7">
         <v>5</v>
       </c>
       <c r="R24" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S24" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="T24" s="7" t="s">
         <v>79</v>
@@ -3457,25 +3603,27 @@
         <v>80</v>
       </c>
       <c r="V24" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="W24" s="9" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
       <c r="X24" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="Y24" s="7"/>
+        <v>249</v>
+      </c>
+      <c r="Y24" s="7" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>228</v>
+        <v>251</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>229</v>
+        <v>252</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="7">
@@ -3488,10 +3636,10 @@
         <v>70</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>230</v>
+        <v>253</v>
       </c>
       <c r="J25" s="8">
         <v>21000</v>
@@ -3503,7 +3651,7 @@
         <v>74</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>231</v>
+        <v>254</v>
       </c>
       <c r="N25" s="7">
         <v>4</v>
@@ -3521,35 +3669,37 @@
         <v>77</v>
       </c>
       <c r="S25" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="T25" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U25" s="7"/>
       <c r="V25" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W25" s="9" t="s">
-        <v>232</v>
+        <v>255</v>
       </c>
       <c r="X25" s="9" t="s">
-        <v>233</v>
-      </c>
-      <c r="Y25" s="7"/>
+        <v>256</v>
+      </c>
+      <c r="Y25" s="7" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>234</v>
+        <v>258</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>235</v>
+        <v>259</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>236</v>
+        <v>260</v>
       </c>
       <c r="E26" s="7">
         <v>2026</v>
@@ -3558,13 +3708,13 @@
         <v>71000000</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J26" s="8">
         <v>0</v>
@@ -3573,23 +3723,23 @@
         <v>73</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>237</v>
+        <v>261</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>238</v>
+        <v>262</v>
       </c>
       <c r="N26" s="7"/>
       <c r="O26" s="7">
         <v>320</v>
       </c>
       <c r="P26" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q26" s="7">
         <v>5</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S26" s="7" t="s">
         <v>78</v>
@@ -3601,19 +3751,21 @@
         <v>80</v>
       </c>
       <c r="V26" s="7" t="s">
-        <v>239</v>
+        <v>263</v>
       </c>
       <c r="W26" s="9" t="s">
-        <v>240</v>
+        <v>264</v>
       </c>
       <c r="X26" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="Y26" s="7"/>
+        <v>265</v>
+      </c>
+      <c r="Y26" s="7" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>242</v>
+        <v>267</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>67</v>
@@ -3622,7 +3774,7 @@
         <v>68</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>243</v>
+        <v>268</v>
       </c>
       <c r="E27" s="7">
         <v>2026</v>
@@ -3631,10 +3783,10 @@
         <v>49000000</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>72</v>
@@ -3646,10 +3798,10 @@
         <v>73</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>244</v>
+        <v>269</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>245</v>
+        <v>270</v>
       </c>
       <c r="N27" s="7">
         <v>4</v>
@@ -3664,38 +3816,40 @@
         <v>5</v>
       </c>
       <c r="R27" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="S27" s="7" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="T27" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U27" s="7"/>
       <c r="V27" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W27" s="9" t="s">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="X27" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="Y27" s="7"/>
+        <v>272</v>
+      </c>
+      <c r="Y27" s="7" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>248</v>
+        <v>274</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>249</v>
+        <v>275</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>251</v>
+        <v>277</v>
       </c>
       <c r="E28" s="7">
         <v>2023</v>
@@ -3722,7 +3876,7 @@
         <v>74</v>
       </c>
       <c r="M28" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N28" s="7">
         <v>4</v>
@@ -3737,10 +3891,10 @@
         <v>5</v>
       </c>
       <c r="R28" s="7" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="S28" s="7" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="T28" s="7" t="s">
         <v>79</v>
@@ -3748,22 +3902,24 @@
       <c r="U28" s="7"/>
       <c r="V28" s="7"/>
       <c r="W28" s="9" t="s">
-        <v>252</v>
+        <v>278</v>
       </c>
       <c r="X28" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="Y28" s="7"/>
+        <v>279</v>
+      </c>
+      <c r="Y28" s="7" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>254</v>
+        <v>281</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>255</v>
+        <v>282</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="7">
@@ -3776,10 +3932,10 @@
         <v>70</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J29" s="8">
         <v>72000</v>
@@ -3791,7 +3947,7 @@
         <v>74</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>257</v>
+        <v>284</v>
       </c>
       <c r="N29" s="7">
         <v>6</v>
@@ -3800,16 +3956,16 @@
         <v>247</v>
       </c>
       <c r="P29" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q29" s="7">
         <v>7</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>258</v>
+        <v>285</v>
       </c>
       <c r="T29" s="7" t="s">
         <v>79</v>
@@ -3817,25 +3973,27 @@
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="9" t="s">
-        <v>259</v>
+        <v>286</v>
       </c>
       <c r="X29" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="Y29" s="7"/>
+        <v>287</v>
+      </c>
+      <c r="Y29" s="7" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>261</v>
+        <v>289</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>262</v>
+        <v>290</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>263</v>
+        <v>291</v>
       </c>
       <c r="E30" s="7">
         <v>2024</v>
@@ -3847,10 +4005,10 @@
         <v>70</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>264</v>
+        <v>292</v>
       </c>
       <c r="J30" s="8">
         <v>26000</v>
@@ -3862,7 +4020,7 @@
         <v>74</v>
       </c>
       <c r="M30" s="7" t="s">
-        <v>265</v>
+        <v>293</v>
       </c>
       <c r="N30" s="7">
         <v>4</v>
@@ -3871,16 +4029,16 @@
         <v>164</v>
       </c>
       <c r="P30" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="Q30" s="7">
         <v>5</v>
       </c>
       <c r="R30" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S30" s="7" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="T30" s="7" t="s">
         <v>79</v>
@@ -3888,22 +4046,24 @@
       <c r="U30" s="7"/>
       <c r="V30" s="7"/>
       <c r="W30" s="9" t="s">
-        <v>266</v>
+        <v>294</v>
       </c>
       <c r="X30" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="Y30" s="7"/>
+        <v>295</v>
+      </c>
+      <c r="Y30" s="7" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>268</v>
+        <v>297</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>269</v>
+        <v>298</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="D31" s="7"/>
       <c r="E31" s="7">
@@ -3913,13 +4073,13 @@
         <v>46000000</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H31" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I31" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="J31" s="8">
         <v>0</v>
@@ -3931,7 +4091,7 @@
         <v>74</v>
       </c>
       <c r="M31" s="7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="N31" s="7">
         <v>4</v>
@@ -3946,7 +4106,7 @@
         <v>5</v>
       </c>
       <c r="R31" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="S31" s="7" t="s">
         <v>78</v>
@@ -3959,22 +4119,24 @@
       </c>
       <c r="V31" s="7"/>
       <c r="W31" s="9" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="X31" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="Y31" s="7"/>
+        <v>301</v>
+      </c>
+      <c r="Y31" s="7" t="s">
+        <v>302</v>
+      </c>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>273</v>
+        <v>303</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>274</v>
+        <v>304</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>275</v>
+        <v>305</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="7">
@@ -3984,13 +4146,13 @@
         <v>34000000</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H32" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I32" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="J32" s="8">
         <v>0</v>
@@ -4002,7 +4164,7 @@
         <v>74</v>
       </c>
       <c r="M32" s="7" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="N32" s="7">
         <v>4</v>
@@ -4020,32 +4182,34 @@
         <v>77</v>
       </c>
       <c r="S32" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="T32" s="7" t="s">
         <v>79</v>
       </c>
       <c r="U32" s="7"/>
       <c r="V32" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="W32" s="9" t="s">
-        <v>276</v>
+        <v>306</v>
       </c>
       <c r="X32" s="9" t="s">
-        <v>277</v>
-      </c>
-      <c r="Y32" s="7"/>
+        <v>307</v>
+      </c>
+      <c r="Y32" s="7" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>278</v>
+        <v>309</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>279</v>
+        <v>310</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>280</v>
+        <v>311</v>
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="7">
@@ -4055,13 +4219,13 @@
         <v>44000000</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H33" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I33" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="J33" s="8">
         <v>0</v>
@@ -4073,7 +4237,7 @@
         <v>74</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="N33" s="7">
         <v>4</v>
@@ -4088,10 +4252,10 @@
         <v>5</v>
       </c>
       <c r="R33" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="S33" s="7" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="T33" s="7" t="s">
         <v>79</v>
@@ -4099,22 +4263,24 @@
       <c r="U33" s="7"/>
       <c r="V33" s="7"/>
       <c r="W33" s="9" t="s">
-        <v>281</v>
+        <v>312</v>
       </c>
       <c r="X33" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="Y33" s="7"/>
+        <v>313</v>
+      </c>
+      <c r="Y33" s="7" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>283</v>
+        <v>315</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>284</v>
+        <v>316</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="7">
@@ -4124,13 +4290,13 @@
         <v>71000000</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="J34" s="8">
         <v>0</v>
@@ -4142,7 +4308,7 @@
         <v>74</v>
       </c>
       <c r="M34" s="7" t="s">
-        <v>285</v>
+        <v>317</v>
       </c>
       <c r="N34" s="7">
         <v>4</v>
@@ -4151,13 +4317,13 @@
         <v>277</v>
       </c>
       <c r="P34" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q34" s="7">
         <v>7</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>286</v>
+        <v>318</v>
       </c>
       <c r="S34" s="7" t="s">
         <v>78</v>
@@ -4170,22 +4336,24 @@
       </c>
       <c r="V34" s="7"/>
       <c r="W34" s="9" t="s">
-        <v>287</v>
+        <v>319</v>
       </c>
       <c r="X34" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="Y34" s="7"/>
+        <v>320</v>
+      </c>
+      <c r="Y34" s="7" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>289</v>
+        <v>322</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>291</v>
+        <v>324</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7">
@@ -4195,13 +4363,13 @@
         <v>48000000</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H35" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I35" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>122</v>
       </c>
       <c r="J35" s="8">
         <v>0</v>
@@ -4213,7 +4381,7 @@
         <v>74</v>
       </c>
       <c r="M35" s="7" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="N35" s="7">
         <v>4</v>
@@ -4222,13 +4390,13 @@
         <v>254</v>
       </c>
       <c r="P35" s="7" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="Q35" s="7">
         <v>7</v>
       </c>
       <c r="R35" s="7" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>78</v>
@@ -4239,12 +4407,14 @@
       <c r="U35" s="7"/>
       <c r="V35" s="7"/>
       <c r="W35" s="9" t="s">
-        <v>292</v>
+        <v>325</v>
       </c>
       <c r="X35" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="Y35" s="7"/>
+        <v>326</v>
+      </c>
+      <c r="Y35" s="7" t="s">
+        <v>327</v>
+      </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
@@ -14223,19 +14393,19 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>294</v>
+        <v>328</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>48</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>295</v>
+        <v>329</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>296</v>
+        <v>330</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>297</v>
+        <v>331</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>56</v>
@@ -14244,7 +14414,7 @@
         <v>58</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>298</v>
+        <v>332</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>60</v>
@@ -14255,10 +14425,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C2" s="11" t="s">
         <v>72</v>
@@ -14273,7 +14443,7 @@
         <v>76</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H2" s="11" t="s">
         <v>78</v>
@@ -14290,31 +14460,31 @@
         <v>70</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>299</v>
+        <v>333</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>300</v>
+        <v>334</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>301</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
@@ -14322,154 +14492,154 @@
         <v>71</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>230</v>
+        <v>253</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>244</v>
+        <v>269</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>302</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>237</v>
+        <v>261</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
-        <v>303</v>
+        <v>337</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>264</v>
+        <v>292</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>77</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
-        <v>304</v>
+        <v>338</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>305</v>
+        <v>339</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>306</v>
+        <v>340</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>307</v>
+        <v>341</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>258</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G9" s="11" t="s">
-        <v>286</v>
+        <v>318</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>308</v>
+        <v>342</v>
       </c>
     </row>
     <row r="10" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G10" s="11" t="s">
-        <v>309</v>
+        <v>343</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>310</v>
+        <v>344</v>
       </c>
     </row>
     <row r="11" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G11" s="11" t="s">
-        <v>311</v>
+        <v>345</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>312</v>
+        <v>346</v>
       </c>
     </row>
     <row r="12" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G12" s="11" t="s">
-        <v>313</v>
+        <v>347</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>314</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G13" s="11" t="s">
-        <v>315</v>
+        <v>349</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>316</v>
+        <v>350</v>
       </c>
     </row>
     <row r="14" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G14" s="11" t="s">
-        <v>317</v>
+        <v>351</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>318</v>
+        <v>352</v>
       </c>
     </row>
     <row r="15" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H15" s="11" t="s">
-        <v>319</v>
+        <v>353</v>
       </c>
     </row>
     <row r="16" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H16" s="11" t="s">
-        <v>320</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H17" s="11" t="s">
-        <v>321</v>
+        <v>355</v>
       </c>
     </row>
     <row r="18" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H18" s="11" t="s">
-        <v>322</v>
+        <v>356</v>
       </c>
     </row>
     <row r="19" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H19" s="11" t="s">
-        <v>323</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Review the downloaded car photos and show them uncropped
- Drop 7 of the 98 photos after looking at each one: another dealer's
  branding on the Defender, right-hand-drive interiors (Defender, Pajero),
  an overhead ES shot, a C 300 d diesel badge, a muddy Prado and Hilux
- Put the clearest front three-quarter photo first for each car, and set
  15 car colours to the colour of that photo
- Show photos whole (object-contain over a blurred copy) in cards and the
  gallery so wide shots keep their bumpers; small thumbnails still fill
- fetch-photos only rewrites cars.xlsx when the photo column changes, so
  the workflow doesn't commit byte-only changes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PG3LFUTwvwMKcvaU6nuHvn
</commit_message>
<xml_diff>
--- a/content/cars.xlsx
+++ b/content/cars.xlsx
@@ -348,271 +348,274 @@
     <t>4.0L V6</t>
   </si>
   <si>
+    <t>أربيل</t>
+  </si>
+  <si>
+    <t>تويوتا برادو TXL 2023 خليجي بمحرك V6 سعة 4.0 لتر، آخر موديل من الجيل المعروف بالمتانة. ممشى 38 ألف كم وصيانة منتظمة، مناسبة للعوائل الكبيرة والسفر.</t>
+  </si>
+  <si>
+    <t>دفع رباعي، سبعة مقاعد، مقاعد جلد، شاشة وسطية، كاميرا خلفية، حساسات ركن أمامية وخلفية</t>
+  </si>
+  <si>
+    <t>car-004-1.webp، car-004-2.webp</t>
+  </si>
+  <si>
+    <t>car-005</t>
+  </si>
+  <si>
+    <t>Kia</t>
+  </si>
+  <si>
+    <t>K5</t>
+  </si>
+  <si>
+    <t>GT-Line</t>
+  </si>
+  <si>
+    <t>كوري</t>
+  </si>
+  <si>
+    <t>1.6L تيربو</t>
+  </si>
+  <si>
+    <t>أزرق</t>
+  </si>
+  <si>
+    <t>كيا K5 GT-Line 2024 وارد كوري بمحرك 1.6 تيربو، تصميم رياضي وتجهيزات كاملة. ممشى 19 ألف كم وحالة شبه جديدة، فخامة بسعر مناسب.</t>
+  </si>
+  <si>
+    <t>شاشة بانورامية مزدوجة، مقاعد جلد مهواة، شاحن لاسلكي، كاميرا خلفية، تحكم مناخي ثنائي، بصمة تشغيل</t>
+  </si>
+  <si>
+    <t>car-005-1.webp، car-005-2.webp، car-005-3.webp</t>
+  </si>
+  <si>
+    <t>car-006</t>
+  </si>
+  <si>
+    <t>Sportage</t>
+  </si>
+  <si>
+    <t>SUV</t>
+  </si>
+  <si>
+    <t>رمادي</t>
+  </si>
+  <si>
+    <t>كيا سبورتاج GT-Line 2023 وارد كوري، الجيل الجديد بالشاشة المنحنية. SUV عملية ومريحة للعائلة، ممشى 27 ألف كم ومساحة داخلية واسعة.</t>
+  </si>
+  <si>
+    <t>شاشة منحنية مزدوجة 12.3 بوصة، فتحة سقف بانورامية، كاميرا خلفية، حساسات ركن، مقاعد جلد، شاحن لاسلكي</t>
+  </si>
+  <si>
+    <t>car-006-1.webp، car-006-2.webp، car-006-3.webp</t>
+  </si>
+  <si>
+    <t>car-007</t>
+  </si>
+  <si>
+    <t>Sorento</t>
+  </si>
+  <si>
+    <t>وكالة</t>
+  </si>
+  <si>
+    <t>3.5L V6</t>
+  </si>
+  <si>
+    <t>كلي</t>
+  </si>
+  <si>
+    <t>كيا سورينتو 2026 وكالة زيرو بمحرك V6 سعة 3.5 لتر ودفع كلي، سبعة مقاعد حقيقية للعوائل الكبيرة. ضمان الوكيل وتجهيزات أمان متقدمة.</t>
+  </si>
+  <si>
+    <t>سبعة مقاعد، دفع كلي AWD، شاشة 12.3 بوصة، كاميرا 360 درجة، مقاعد جلد، فتحة سقف بانورامية، ضمان الوكيل</t>
+  </si>
+  <si>
+    <t>car-007-1.webp، car-007-2.webp، car-007-3.webp</t>
+  </si>
+  <si>
+    <t>car-008</t>
+  </si>
+  <si>
+    <t>Hyundai</t>
+  </si>
+  <si>
+    <t>Sonata</t>
+  </si>
+  <si>
+    <t>هيونداي سوناتا 2023 وارد كوري، سيدان عائلية واسعة وهادئة. ممشى 41 ألف كم وسجل صيانة واضح.</t>
+  </si>
+  <si>
+    <t>شاشة 10.25 بوصة، كاميرا خلفية، بلوتوث، تحكم مناخي، مقاعد مدفأة</t>
+  </si>
+  <si>
+    <t>car-008-1.webp، car-008-2.webp، car-008-3.webp</t>
+  </si>
+  <si>
+    <t>car-009</t>
+  </si>
+  <si>
+    <t>Tucson</t>
+  </si>
+  <si>
+    <t>النجف</t>
+  </si>
+  <si>
+    <t>هيونداي توسان 2024 خليجي بالتصميم المحدّث، ممشى 14 ألف كم وحالة قريبة من الجديدة. تجهيزات تقنية متقدمة واستهلاك وقود معتدل.</t>
+  </si>
+  <si>
+    <t>شاشة 12.3 بوصة، كاميرا خلفية، حساسات ركن، مقاعد جلد، تحكم مناخي أوتوماتيك، مثبت سرعة</t>
+  </si>
+  <si>
+    <t>car-009-1.webp، car-009-2.webp، car-009-3.webp</t>
+  </si>
+  <si>
+    <t>car-010</t>
+  </si>
+  <si>
+    <t>Elantra</t>
+  </si>
+  <si>
+    <t>SEL</t>
+  </si>
+  <si>
+    <t>كربلاء</t>
+  </si>
+  <si>
+    <t>هيونداي إلنترا SEL 2023 وارد أمريكي، خيار اقتصادي وعملي للاستخدام اليومي. ممشى 36 ألف كم وحالة ميكانيكية ممتازة.</t>
+  </si>
+  <si>
+    <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، مثبت سرعة، تنبيه النقطة العمياء</t>
+  </si>
+  <si>
+    <t>car-010-1.webp، car-010-2.webp</t>
+  </si>
+  <si>
+    <t>car-011</t>
+  </si>
+  <si>
+    <t>Nissan</t>
+  </si>
+  <si>
+    <t>Altima</t>
+  </si>
+  <si>
+    <t>SV</t>
+  </si>
+  <si>
+    <t>محجوزة</t>
+  </si>
+  <si>
+    <t>نيسان التيما SV 2023 وارد أمريكي، مريحة وهادئة القيادة مع استهلاك وقود معقول. ممشى 31 ألف كم وحالة نظيفة جداً.</t>
+  </si>
+  <si>
+    <t>شاشة 8 بوصة، كاميرا خلفية، مثبت سرعة تكيفي ProPilot، مقاعد مدفأة، تشغيل بدون مفتاح</t>
+  </si>
+  <si>
+    <t>car-011-1.webp، car-011-2.webp، car-011-3.webp</t>
+  </si>
+  <si>
+    <t>car-012</t>
+  </si>
+  <si>
+    <t>Patrol</t>
+  </si>
+  <si>
+    <t>LE Platinum</t>
+  </si>
+  <si>
+    <t>نيسان باترول LE بلاتينيوم 2026 خليجي زيرو، الجيل الجديد بمحرك V6 توين تيربو بقوة 425 حصان. فخامة كاملة ومقصورة واسعة لثمانية ركاب، رمز القوة في السوق العراقي.</t>
+  </si>
+  <si>
+    <t>شاشتان 14.3 بوصة، كاميرا 360 درجة، تعليق هوائي، مقاعد جلد مدفأة ومهواة، نظام صوت Klipsch، فتحة سقف بانورامية، ثمانية مقاعد</t>
+  </si>
+  <si>
+    <t>car-012-1.webp، car-012-2.webp، car-012-3.webp</t>
+  </si>
+  <si>
+    <t>car-013</t>
+  </si>
+  <si>
+    <t>Sunny</t>
+  </si>
+  <si>
+    <t>1.6L</t>
+  </si>
+  <si>
+    <t>الموصل</t>
+  </si>
+  <si>
+    <t>نيسان صني 2024 وكالة، من أكثر السيارات اقتصادية بالوقود والصيانة. ممشى 22 ألف كم، خيار موثوق لأول سيارة ولسائقي التطبيقات.</t>
+  </si>
+  <si>
+    <t>شاشة وسطية، بلوتوث، كاميرا خلفية، مكيف أوتوماتيك</t>
+  </si>
+  <si>
+    <t>car-013-1.webp، car-013-2.webp، car-013-3.webp</t>
+  </si>
+  <si>
+    <t>car-014</t>
+  </si>
+  <si>
+    <t>Chevrolet</t>
+  </si>
+  <si>
+    <t>Malibu</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>1.5L تيربو</t>
+  </si>
+  <si>
+    <t>شفروليه ماليبو LT 2023 وارد أمريكي، من أكثر السيارات انتشاراً في العراق لراحتها ومساحتها الداخلية الواسعة. ممشى 44 ألف كم.</t>
+  </si>
+  <si>
+    <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، تشغيل عن بعد، مقاعد قماش فاخر</t>
+  </si>
+  <si>
+    <t>car-014-1.webp، car-014-2.webp</t>
+  </si>
+  <si>
+    <t>car-015</t>
+  </si>
+  <si>
+    <t>Tahoe</t>
+  </si>
+  <si>
+    <t>5.3L V8</t>
+  </si>
+  <si>
+    <t>شفروليه تاهو LT 2023 وارد أمريكي بمحرك V8 ودفع رباعي، SUV كبيرة تتسع لثمانية ركاب براحة تامة. ممشى 33 ألف كم.</t>
+  </si>
+  <si>
+    <t>ثمانية مقاعد، دفع رباعي، شاشة 10.2 بوصة، مقاعد جلد، كاميرا خلفية، تشغيل عن بعد</t>
+  </si>
+  <si>
+    <t>car-015-1.webp، car-015-2.webp، car-015-3.webp</t>
+  </si>
+  <si>
+    <t>car-016</t>
+  </si>
+  <si>
+    <t>Lexus</t>
+  </si>
+  <si>
+    <t>ES 350</t>
+  </si>
+  <si>
     <t>فضي</t>
   </si>
   <si>
-    <t>أربيل</t>
-  </si>
-  <si>
-    <t>تويوتا برادو TXL 2023 خليجي بمحرك V6 سعة 4.0 لتر، آخر موديل من الجيل المعروف بالمتانة. ممشى 38 ألف كم وصيانة منتظمة، مناسبة للعوائل الكبيرة والسفر.</t>
-  </si>
-  <si>
-    <t>دفع رباعي، سبعة مقاعد، مقاعد جلد، شاشة وسطية، كاميرا خلفية، حساسات ركن أمامية وخلفية</t>
-  </si>
-  <si>
-    <t>car-004-1.webp، car-004-2.webp، car-004-3.webp</t>
-  </si>
-  <si>
-    <t>car-005</t>
-  </si>
-  <si>
-    <t>Kia</t>
-  </si>
-  <si>
-    <t>K5</t>
-  </si>
-  <si>
-    <t>GT-Line</t>
-  </si>
-  <si>
-    <t>كوري</t>
-  </si>
-  <si>
-    <t>1.6L تيربو</t>
-  </si>
-  <si>
-    <t>رمادي</t>
-  </si>
-  <si>
-    <t>كيا K5 GT-Line 2024 وارد كوري بمحرك 1.6 تيربو، تصميم رياضي وتجهيزات كاملة. ممشى 19 ألف كم وحالة شبه جديدة، فخامة بسعر مناسب.</t>
-  </si>
-  <si>
-    <t>شاشة بانورامية مزدوجة، مقاعد جلد مهواة، شاحن لاسلكي، كاميرا خلفية، تحكم مناخي ثنائي، بصمة تشغيل</t>
-  </si>
-  <si>
-    <t>car-005-1.webp، car-005-2.webp، car-005-3.webp</t>
-  </si>
-  <si>
-    <t>car-006</t>
-  </si>
-  <si>
-    <t>Sportage</t>
-  </si>
-  <si>
-    <t>SUV</t>
-  </si>
-  <si>
-    <t>كيا سبورتاج GT-Line 2023 وارد كوري، الجيل الجديد بالشاشة المنحنية. SUV عملية ومريحة للعائلة، ممشى 27 ألف كم ومساحة داخلية واسعة.</t>
-  </si>
-  <si>
-    <t>شاشة منحنية مزدوجة 12.3 بوصة، فتحة سقف بانورامية، كاميرا خلفية، حساسات ركن، مقاعد جلد، شاحن لاسلكي</t>
-  </si>
-  <si>
-    <t>car-006-1.webp، car-006-2.webp، car-006-3.webp</t>
-  </si>
-  <si>
-    <t>car-007</t>
-  </si>
-  <si>
-    <t>Sorento</t>
-  </si>
-  <si>
-    <t>وكالة</t>
-  </si>
-  <si>
-    <t>3.5L V6</t>
-  </si>
-  <si>
-    <t>كلي</t>
-  </si>
-  <si>
-    <t>كيا سورينتو 2026 وكالة زيرو بمحرك V6 سعة 3.5 لتر ودفع كلي، سبعة مقاعد حقيقية للعوائل الكبيرة. ضمان الوكيل وتجهيزات أمان متقدمة.</t>
-  </si>
-  <si>
-    <t>سبعة مقاعد، دفع كلي AWD، شاشة 12.3 بوصة، كاميرا 360 درجة، مقاعد جلد، فتحة سقف بانورامية، ضمان الوكيل</t>
-  </si>
-  <si>
-    <t>car-007-1.webp، car-007-2.webp، car-007-3.webp</t>
-  </si>
-  <si>
-    <t>car-008</t>
-  </si>
-  <si>
-    <t>Hyundai</t>
-  </si>
-  <si>
-    <t>Sonata</t>
-  </si>
-  <si>
-    <t>هيونداي سوناتا 2023 وارد كوري، سيدان عائلية واسعة وهادئة. ممشى 41 ألف كم وسجل صيانة واضح.</t>
-  </si>
-  <si>
-    <t>شاشة 10.25 بوصة، كاميرا خلفية، بلوتوث، تحكم مناخي، مقاعد مدفأة</t>
-  </si>
-  <si>
-    <t>car-008-1.webp، car-008-2.webp، car-008-3.webp</t>
-  </si>
-  <si>
-    <t>car-009</t>
-  </si>
-  <si>
-    <t>Tucson</t>
-  </si>
-  <si>
-    <t>النجف</t>
-  </si>
-  <si>
-    <t>هيونداي توسان 2024 خليجي بالتصميم المحدّث، ممشى 14 ألف كم وحالة قريبة من الجديدة. تجهيزات تقنية متقدمة واستهلاك وقود معتدل.</t>
-  </si>
-  <si>
-    <t>شاشة 12.3 بوصة، كاميرا خلفية، حساسات ركن، مقاعد جلد، تحكم مناخي أوتوماتيك، مثبت سرعة</t>
-  </si>
-  <si>
-    <t>car-009-1.webp، car-009-2.webp، car-009-3.webp</t>
-  </si>
-  <si>
-    <t>car-010</t>
-  </si>
-  <si>
-    <t>Elantra</t>
-  </si>
-  <si>
-    <t>SEL</t>
-  </si>
-  <si>
-    <t>كربلاء</t>
-  </si>
-  <si>
-    <t>هيونداي إلنترا SEL 2023 وارد أمريكي، خيار اقتصادي وعملي للاستخدام اليومي. ممشى 36 ألف كم وحالة ميكانيكية ممتازة.</t>
-  </si>
-  <si>
-    <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، مثبت سرعة، تنبيه النقطة العمياء</t>
-  </si>
-  <si>
-    <t>car-010-1.webp، car-010-2.webp</t>
-  </si>
-  <si>
-    <t>car-011</t>
-  </si>
-  <si>
-    <t>Nissan</t>
-  </si>
-  <si>
-    <t>Altima</t>
-  </si>
-  <si>
-    <t>SV</t>
-  </si>
-  <si>
-    <t>محجوزة</t>
-  </si>
-  <si>
-    <t>نيسان التيما SV 2023 وارد أمريكي، مريحة وهادئة القيادة مع استهلاك وقود معقول. ممشى 31 ألف كم وحالة نظيفة جداً.</t>
-  </si>
-  <si>
-    <t>شاشة 8 بوصة، كاميرا خلفية، مثبت سرعة تكيفي ProPilot، مقاعد مدفأة، تشغيل بدون مفتاح</t>
-  </si>
-  <si>
-    <t>car-011-1.webp، car-011-2.webp، car-011-3.webp</t>
-  </si>
-  <si>
-    <t>car-012</t>
-  </si>
-  <si>
-    <t>Patrol</t>
-  </si>
-  <si>
-    <t>LE Platinum</t>
-  </si>
-  <si>
-    <t>نيسان باترول LE بلاتينيوم 2026 خليجي زيرو، الجيل الجديد بمحرك V6 توين تيربو بقوة 425 حصان. فخامة كاملة ومقصورة واسعة لثمانية ركاب، رمز القوة في السوق العراقي.</t>
-  </si>
-  <si>
-    <t>شاشتان 14.3 بوصة، كاميرا 360 درجة، تعليق هوائي، مقاعد جلد مدفأة ومهواة، نظام صوت Klipsch، فتحة سقف بانورامية، ثمانية مقاعد</t>
-  </si>
-  <si>
-    <t>car-012-1.webp، car-012-2.webp، car-012-3.webp</t>
-  </si>
-  <si>
-    <t>car-013</t>
-  </si>
-  <si>
-    <t>Sunny</t>
-  </si>
-  <si>
-    <t>1.6L</t>
-  </si>
-  <si>
-    <t>الموصل</t>
-  </si>
-  <si>
-    <t>نيسان صني 2024 وكالة، من أكثر السيارات اقتصادية بالوقود والصيانة. ممشى 22 ألف كم، خيار موثوق لأول سيارة ولسائقي التطبيقات.</t>
-  </si>
-  <si>
-    <t>شاشة وسطية، بلوتوث، كاميرا خلفية، مكيف أوتوماتيك</t>
-  </si>
-  <si>
-    <t>car-013-1.webp، car-013-2.webp، car-013-3.webp</t>
-  </si>
-  <si>
-    <t>car-014</t>
-  </si>
-  <si>
-    <t>Chevrolet</t>
-  </si>
-  <si>
-    <t>Malibu</t>
-  </si>
-  <si>
-    <t>LT</t>
-  </si>
-  <si>
-    <t>1.5L تيربو</t>
-  </si>
-  <si>
-    <t>شفروليه ماليبو LT 2023 وارد أمريكي، من أكثر السيارات انتشاراً في العراق لراحتها ومساحتها الداخلية الواسعة. ممشى 44 ألف كم.</t>
-  </si>
-  <si>
-    <t>شاشة 8 بوصة، آبل كاربلاي، كاميرا خلفية، تشغيل عن بعد، مقاعد قماش فاخر</t>
-  </si>
-  <si>
-    <t>car-014-1.webp، car-014-2.webp</t>
-  </si>
-  <si>
-    <t>car-015</t>
-  </si>
-  <si>
-    <t>Tahoe</t>
-  </si>
-  <si>
-    <t>5.3L V8</t>
-  </si>
-  <si>
-    <t>شفروليه تاهو LT 2023 وارد أمريكي بمحرك V8 ودفع رباعي، SUV كبيرة تتسع لثمانية ركاب براحة تامة. ممشى 33 ألف كم.</t>
-  </si>
-  <si>
-    <t>ثمانية مقاعد، دفع رباعي، شاشة 10.2 بوصة، مقاعد جلد، كاميرا خلفية، تشغيل عن بعد</t>
-  </si>
-  <si>
-    <t>car-015-1.webp، car-015-2.webp، car-015-3.webp</t>
-  </si>
-  <si>
-    <t>car-016</t>
-  </si>
-  <si>
-    <t>Lexus</t>
-  </si>
-  <si>
-    <t>ES 350</t>
-  </si>
-  <si>
     <t>لكزس ES 350 2023 وارد أمريكي، فخامة يابانية هادئة مع عزل صوت ممتاز وراحة قيادة عالية. ممشى 24 ألف كم وصيانة منتظمة.</t>
   </si>
   <si>
     <t>مقاعد جلد مدفأة ومهواة، فتحة سقف، نظام صوت مارك ليفنسون، شاشة 12.3 بوصة، كاميرا خلفية، حساسات ركن</t>
   </si>
   <si>
-    <t>car-016-1.webp، car-016-2.webp، car-016-3.webp</t>
+    <t>car-016-1.webp، car-016-2.webp</t>
   </si>
   <si>
     <t>car-017</t>
@@ -624,9 +627,6 @@
     <t>2.4L تيربو</t>
   </si>
   <si>
-    <t>أزرق</t>
-  </si>
-  <si>
     <t>لكزس RX 350 2024 خليجي، الجيل الجديد بمحرك 2.4 تيربو ودفع كلي. SUV فاخرة بتصميم جريء وتجهيزات أمان متقدمة، بحالة ممتازة.</t>
   </si>
   <si>
@@ -660,7 +660,7 @@
     <t>شاشة MBUX 11.9 بوصة، مقاعد جلد مدفأة، كاميرا 360 درجة، إضاءة أمبيانت، فتحة سقف بانورامية</t>
   </si>
   <si>
-    <t>car-018-1.webp، car-018-2.webp، car-018-3.webp</t>
+    <t>car-018-1.webp، car-018-2.webp</t>
   </si>
   <si>
     <t>car-019</t>
@@ -762,13 +762,16 @@
     <t>110 X-Dynamic SE</t>
   </si>
   <si>
+    <t>أخضر</t>
+  </si>
+  <si>
     <t>لاند روفر ديفندر 110 موديل 2024 خليجي، تصميم عصري بروح مغامرة وقدرات عبور استثنائية مع فخامة داخلية. ممشى 12 ألف كم.</t>
   </si>
   <si>
     <t>دفع كلي مع تعليق هوائي، شاشة Pivi Pro 11.4 بوصة، كاميرا 360 درجة، مقاعد جلد، نظام Terrain Response</t>
   </si>
   <si>
-    <t>car-023-1.webp، car-023-2.webp، car-023-3.webp</t>
+    <t>car-023-1.webp</t>
   </si>
   <si>
     <t>car-024</t>
@@ -882,7 +885,7 @@
     <t>دفع رباعي Super Select، سبعة مقاعد، شاشة وسطية، كاميرا خلفية، مقاعد جلد</t>
   </si>
   <si>
-    <t>car-028-1.webp، car-028-2.webp، car-028-3.webp</t>
+    <t>car-028-1.webp، car-028-2.webp</t>
   </si>
   <si>
     <t>car-029</t>
@@ -906,7 +909,7 @@
     <t>دفع رباعي، صندوق خلفي، شاشة 8 بوصة، كاميرا خلفية، مثبت سرعة</t>
   </si>
   <si>
-    <t>car-029-1.webp، car-029-2.webp، car-029-3.webp</t>
+    <t>car-029-1.webp، car-029-2.webp</t>
   </si>
   <si>
     <t>car-030</t>
@@ -954,6 +957,9 @@
     <t>H6</t>
   </si>
   <si>
+    <t>بيج</t>
+  </si>
+  <si>
     <t>هافال H6 2026 وكالة زيرو، SUV عائلية واسعة بمحرك 2.0 تيربو وتجهيزات تقنية متقدمة، مع ضمان الوكيل.</t>
   </si>
   <si>
@@ -972,9 +978,6 @@
     <t>2.5L تيربو</t>
   </si>
   <si>
-    <t>أخضر</t>
-  </si>
-  <si>
     <t>هيونداي سنتافي 2026 خليجي زيرو، الجيل الجديد بالتصميم المربع الواسع وسبعة مقاعد. محرك 2.5 تيربو ودفع كلي، خيار مثالي للعائلة الكبيرة.</t>
   </si>
   <si>
@@ -1051,9 +1054,6 @@
   </si>
   <si>
     <t>كركوك</t>
-  </si>
-  <si>
-    <t>بيج</t>
   </si>
   <si>
     <t>الحلة</t>
@@ -2176,10 +2176,10 @@
         <v>7</v>
       </c>
       <c r="R5" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="S5" s="7" t="s">
         <v>110</v>
-      </c>
-      <c r="S5" s="7" t="s">
-        <v>111</v>
       </c>
       <c r="T5" s="7" t="s">
         <v>79</v>
@@ -2187,27 +2187,27 @@
       <c r="U5" s="7"/>
       <c r="V5" s="7"/>
       <c r="W5" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="X5" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="X5" s="9" t="s">
+      <c r="Y5" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="Y5" s="7" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>117</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>118</v>
       </c>
       <c r="E6" s="7">
         <v>2024</v>
@@ -2219,7 +2219,7 @@
         <v>70</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>72</v>
@@ -2234,7 +2234,7 @@
         <v>74</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N6" s="7">
         <v>4</v>
@@ -2249,7 +2249,7 @@
         <v>5</v>
       </c>
       <c r="R6" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="S6" s="7" t="s">
         <v>78</v>
@@ -2262,27 +2262,27 @@
       </c>
       <c r="V6" s="7"/>
       <c r="W6" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="X6" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="X6" s="9" t="s">
+      <c r="Y6" s="7" t="s">
         <v>123</v>
-      </c>
-      <c r="Y6" s="7" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>126</v>
-      </c>
       <c r="D7" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E7" s="7">
         <v>2023</v>
@@ -2294,10 +2294,10 @@
         <v>70</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J7" s="8">
         <v>27000</v>
@@ -2309,7 +2309,7 @@
         <v>74</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N7" s="7">
         <v>4</v>
@@ -2324,10 +2324,10 @@
         <v>5</v>
       </c>
       <c r="R7" s="7" t="s">
-        <v>101</v>
+        <v>127</v>
       </c>
       <c r="S7" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T7" s="7" t="s">
         <v>79</v>
@@ -2351,7 +2351,7 @@
         <v>131</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>132</v>
@@ -2370,7 +2370,7 @@
         <v>133</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
@@ -2397,7 +2397,7 @@
         <v>7</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="S8" s="7" t="s">
         <v>78</v>
@@ -2438,7 +2438,7 @@
         <v>70</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>72</v>
@@ -2468,7 +2468,7 @@
         <v>5</v>
       </c>
       <c r="R9" s="7" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="S9" s="7" t="s">
         <v>78</v>
@@ -2512,7 +2512,7 @@
         <v>97</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J10" s="8">
         <v>14000</v>
@@ -2614,7 +2614,7 @@
         <v>5</v>
       </c>
       <c r="R11" s="7" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="S11" s="7" t="s">
         <v>154</v>
@@ -2912,7 +2912,7 @@
         <v>5</v>
       </c>
       <c r="R15" s="7" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="S15" s="7" t="s">
         <v>78</v>
@@ -2960,7 +2960,7 @@
         <v>71</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J16" s="8">
         <v>33000</v>
@@ -3060,7 +3060,7 @@
         <v>5</v>
       </c>
       <c r="R17" s="7" t="s">
-        <v>87</v>
+        <v>196</v>
       </c>
       <c r="S17" s="7" t="s">
         <v>78</v>
@@ -3075,24 +3075,24 @@
         <v>102</v>
       </c>
       <c r="W17" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="X17" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Y17" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>194</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="7">
@@ -3108,7 +3108,7 @@
         <v>97</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J18" s="8">
         <v>15000</v>
@@ -3120,7 +3120,7 @@
         <v>74</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N18" s="7">
         <v>4</v>
@@ -3135,10 +3135,10 @@
         <v>5</v>
       </c>
       <c r="R18" s="7" t="s">
-        <v>202</v>
+        <v>77</v>
       </c>
       <c r="S18" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T18" s="7" t="s">
         <v>79</v>
@@ -3260,7 +3260,7 @@
         <v>97</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J20" s="8">
         <v>0</v>
@@ -3287,7 +3287,7 @@
         <v>5</v>
       </c>
       <c r="R20" s="7" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="S20" s="7" t="s">
         <v>78</v>
@@ -3367,7 +3367,7 @@
         <v>87</v>
       </c>
       <c r="S21" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T21" s="7" t="s">
         <v>79</v>
@@ -3414,7 +3414,7 @@
         <v>97</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J22" s="8">
         <v>0</v>
@@ -3491,7 +3491,7 @@
         <v>71</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J23" s="8">
         <v>58000</v>
@@ -3591,10 +3591,10 @@
         <v>5</v>
       </c>
       <c r="R24" s="7" t="s">
-        <v>87</v>
+        <v>248</v>
       </c>
       <c r="S24" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T24" s="7" t="s">
         <v>79</v>
@@ -3606,24 +3606,24 @@
         <v>102</v>
       </c>
       <c r="W24" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="X24" s="9" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="Y24" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="7">
@@ -3639,7 +3639,7 @@
         <v>133</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J25" s="8">
         <v>21000</v>
@@ -3651,7 +3651,7 @@
         <v>74</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="N25" s="7">
         <v>4</v>
@@ -3666,7 +3666,7 @@
         <v>5</v>
       </c>
       <c r="R25" s="7" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="S25" s="7" t="s">
         <v>88</v>
@@ -3679,27 +3679,27 @@
         <v>89</v>
       </c>
       <c r="W25" s="9" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="X25" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="Y25" s="7" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E26" s="7">
         <v>2026</v>
@@ -3711,10 +3711,10 @@
         <v>96</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J26" s="8">
         <v>0</v>
@@ -3723,10 +3723,10 @@
         <v>73</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M26" s="7" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N26" s="7"/>
       <c r="O26" s="7">
@@ -3739,7 +3739,7 @@
         <v>5</v>
       </c>
       <c r="R26" s="7" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="S26" s="7" t="s">
         <v>78</v>
@@ -3751,21 +3751,21 @@
         <v>80</v>
       </c>
       <c r="V26" s="7" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="W26" s="9" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="X26" s="9" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Y26" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>67</v>
@@ -3774,7 +3774,7 @@
         <v>68</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E27" s="7">
         <v>2026</v>
@@ -3798,10 +3798,10 @@
         <v>73</v>
       </c>
       <c r="L27" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="M27" s="7" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N27" s="7">
         <v>4</v>
@@ -3816,7 +3816,7 @@
         <v>5</v>
       </c>
       <c r="R27" s="7" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="S27" s="7" t="s">
         <v>154</v>
@@ -3829,27 +3829,27 @@
         <v>89</v>
       </c>
       <c r="W27" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="X27" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Y27" s="7" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E28" s="7">
         <v>2023</v>
@@ -3891,7 +3891,7 @@
         <v>5</v>
       </c>
       <c r="R28" s="7" t="s">
-        <v>202</v>
+        <v>120</v>
       </c>
       <c r="S28" s="7" t="s">
         <v>175</v>
@@ -3902,24 +3902,24 @@
       <c r="U28" s="7"/>
       <c r="V28" s="7"/>
       <c r="W28" s="9" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="X28" s="9" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Y28" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="7">
@@ -3947,7 +3947,7 @@
         <v>74</v>
       </c>
       <c r="M29" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="N29" s="7">
         <v>6</v>
@@ -3962,10 +3962,10 @@
         <v>7</v>
       </c>
       <c r="R29" s="7" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="S29" s="7" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="T29" s="7" t="s">
         <v>79</v>
@@ -3973,27 +3973,27 @@
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="X29" s="9" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="Y29" s="7" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B30" s="7" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E30" s="7">
         <v>2024</v>
@@ -4008,7 +4008,7 @@
         <v>97</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J30" s="8">
         <v>26000</v>
@@ -4020,7 +4020,7 @@
         <v>74</v>
       </c>
       <c r="M30" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="N30" s="7">
         <v>4</v>
@@ -4046,24 +4046,24 @@
       <c r="U30" s="7"/>
       <c r="V30" s="7"/>
       <c r="W30" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="X30" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Y30" s="7" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D31" s="7"/>
       <c r="E31" s="7">
@@ -4079,7 +4079,7 @@
         <v>133</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J31" s="8">
         <v>0</v>
@@ -4106,7 +4106,7 @@
         <v>5</v>
       </c>
       <c r="R31" s="7" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="S31" s="7" t="s">
         <v>78</v>
@@ -4119,24 +4119,24 @@
       </c>
       <c r="V31" s="7"/>
       <c r="W31" s="9" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="X31" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="Y31" s="7" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D32" s="7"/>
       <c r="E32" s="7">
@@ -4152,7 +4152,7 @@
         <v>133</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J32" s="8">
         <v>0</v>
@@ -4179,7 +4179,7 @@
         <v>5</v>
       </c>
       <c r="R32" s="7" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="S32" s="7" t="s">
         <v>88</v>
@@ -4192,24 +4192,24 @@
         <v>89</v>
       </c>
       <c r="W32" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="X32" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="Y32" s="7" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="7">
@@ -4225,7 +4225,7 @@
         <v>133</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J33" s="8">
         <v>0</v>
@@ -4252,10 +4252,10 @@
         <v>5</v>
       </c>
       <c r="R33" s="7" t="s">
-        <v>87</v>
+        <v>313</v>
       </c>
       <c r="S33" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="T33" s="7" t="s">
         <v>79</v>
@@ -4263,24 +4263,24 @@
       <c r="U33" s="7"/>
       <c r="V33" s="7"/>
       <c r="W33" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="X33" s="9" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="Y33" s="7" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>140</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="7">
@@ -4296,7 +4296,7 @@
         <v>97</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J34" s="8">
         <v>0</v>
@@ -4308,7 +4308,7 @@
         <v>74</v>
       </c>
       <c r="M34" s="7" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="N34" s="7">
         <v>4</v>
@@ -4323,7 +4323,7 @@
         <v>7</v>
       </c>
       <c r="R34" s="7" t="s">
-        <v>318</v>
+        <v>248</v>
       </c>
       <c r="S34" s="7" t="s">
         <v>78</v>
@@ -4336,24 +4336,24 @@
       </c>
       <c r="V34" s="7"/>
       <c r="W34" s="9" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="X34" s="9" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Y34" s="7" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="7">
@@ -4369,7 +4369,7 @@
         <v>133</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J35" s="8">
         <v>0</v>
@@ -4396,7 +4396,7 @@
         <v>7</v>
       </c>
       <c r="R35" s="7" t="s">
-        <v>110</v>
+        <v>87</v>
       </c>
       <c r="S35" s="7" t="s">
         <v>78</v>
@@ -4407,13 +4407,13 @@
       <c r="U35" s="7"/>
       <c r="V35" s="7"/>
       <c r="W35" s="9" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="X35" s="9" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="Y35" s="7" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
@@ -14393,19 +14393,19 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>48</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>56</v>
@@ -14414,7 +14414,7 @@
         <v>58</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>60</v>
@@ -14463,13 +14463,13 @@
         <v>97</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F3" s="11" t="s">
         <v>211</v>
@@ -14484,7 +14484,7 @@
         <v>162</v>
       </c>
       <c r="J3" s="11" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
@@ -14492,50 +14492,50 @@
         <v>71</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>100</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>110</v>
+        <v>196</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>175</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>98</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>135</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>77</v>
@@ -14546,13 +14546,13 @@
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="11" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>202</v>
+        <v>120</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>154</v>
@@ -14560,34 +14560,34 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G9" s="11" t="s">
-        <v>318</v>
+        <v>248</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G10" s="11" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G11" s="11" t="s">
-        <v>345</v>
+        <v>313</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>346</v>

</xml_diff>